<commit_message>
database changes, UI and UX changes
</commit_message>
<xml_diff>
--- a/Clase_2_2026-02-06.xlsx
+++ b/Clase_2_2026-02-06.xlsx
@@ -463,7 +463,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>No asistió</t>
+          <t>Asistió</t>
         </is>
       </c>
     </row>
@@ -480,7 +480,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>54.31%</t>
+          <t>57.91%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">

</xml_diff>